<commit_message>
Add Adaa (₹5,499), update all product descriptions with Why You'll Love It
</commit_message>
<xml_diff>
--- a/business/inventory-ledger.xlsx
+++ b/business/inventory-ledger.xlsx
@@ -8,19 +8,32 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ahujadiv\Desktop\Team\Automations\JBG\jewels-by-geetika\business\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B14F6945-E881-4364-9951-0796CF360D85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0685FC22-A4DD-4839-9141-6A71432F6149}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{68BF2D20-07EA-4E2C-B5AF-3720521CC247}"/>
   </bookViews>
   <sheets>
     <sheet name="inventory-ledger" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="39">
   <si>
     <t>Product ID</t>
   </si>
@@ -88,9 +101,6 @@
     <t>JBG-001</t>
   </si>
   <si>
-    <t>Kaveri Necklace Set</t>
-  </si>
-  <si>
     <t>Necklaces</t>
   </si>
   <si>
@@ -115,9 +125,6 @@
     <t>JBG-002</t>
   </si>
   <si>
-    <t>Raahi Necklace Set</t>
-  </si>
-  <si>
     <t>JBG-NCK-002</t>
   </si>
   <si>
@@ -131,6 +138,18 @@
   </si>
   <si>
     <t>JBG-005</t>
+  </si>
+  <si>
+    <t>Kaveri</t>
+  </si>
+  <si>
+    <t>Raahi</t>
+  </si>
+  <si>
+    <t>Saanjh</t>
+  </si>
+  <si>
+    <t>Adaa</t>
   </si>
 </sst>
 </file>
@@ -620,13 +639,16 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="42">
@@ -1078,14 +1100,14 @@
       <c r="A2" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="D2" s="1" t="s">
         <v>23</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>24</v>
       </c>
       <c r="E2" s="1">
         <v>450</v>
@@ -1112,39 +1134,39 @@
         <v>2</v>
       </c>
       <c r="N2" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="O2" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="O2" s="1" t="s">
+      <c r="Q2" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="Q2" s="1" t="s">
+      <c r="R2" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="R2" s="1" t="s">
+      <c r="S2" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="T2" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="U2" s="1" t="s">
         <v>28</v>
-      </c>
-      <c r="S2" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="T2" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="U2" s="1" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="3" spans="1:21" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>31</v>
+        <v>29</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>36</v>
       </c>
       <c r="C3" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D3" s="1" t="s">
         <v>23</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>24</v>
       </c>
       <c r="E3" s="1">
         <v>1240</v>
@@ -1171,40 +1193,70 @@
         <v>2</v>
       </c>
       <c r="N3" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="O3" s="1" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="Q3" s="1" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="R3" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="S3" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="T3" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="U3" s="1" t="s">
         <v>28</v>
-      </c>
-      <c r="S3" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="T3" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="U3" s="1" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="4" spans="1:21" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>34</v>
+        <v>32</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="E4" s="1">
+        <v>1495</v>
+      </c>
+      <c r="H4" s="1">
+        <v>1415</v>
+      </c>
+      <c r="I4" s="1">
+        <v>5</v>
+      </c>
+      <c r="J4" s="1">
+        <v>3499</v>
       </c>
     </row>
     <row r="5" spans="1:21" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>35</v>
+        <v>33</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="E5" s="1">
+        <v>1134</v>
+      </c>
+      <c r="H5" s="1">
+        <v>1415</v>
+      </c>
+      <c r="I5" s="1">
+        <v>5</v>
+      </c>
+      <c r="J5" s="1">
+        <v>3499</v>
       </c>
     </row>
     <row r="6" spans="1:21" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Separate Why You'll Love It into highlighted gold box on product page
</commit_message>
<xml_diff>
--- a/business/inventory-ledger.xlsx
+++ b/business/inventory-ledger.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ahujadiv\Desktop\Team\Automations\JBG\jewels-by-geetika\business\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0685FC22-A4DD-4839-9141-6A71432F6149}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD8B8C02-F650-45C3-84B8-31935A18E0E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{68BF2D20-07EA-4E2C-B5AF-3720521CC247}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="47">
   <si>
     <t>Product ID</t>
   </si>
@@ -113,9 +113,6 @@
     <t>JBG-NCK-001</t>
   </si>
   <si>
-    <t>Kundan + Gold Plating</t>
-  </si>
-  <si>
     <t>Yes</t>
   </si>
   <si>
@@ -128,9 +125,6 @@
     <t>JBG-NCK-002</t>
   </si>
   <si>
-    <t>Polki + Pearl + Pink Beads</t>
-  </si>
-  <si>
     <t>JBG-003</t>
   </si>
   <si>
@@ -150,6 +144,36 @@
   </si>
   <si>
     <t>Adaa</t>
+  </si>
+  <si>
+    <t>AD - Pendant</t>
+  </si>
+  <si>
+    <t>JBG-NCK-003</t>
+  </si>
+  <si>
+    <t>JBG-ADP-001</t>
+  </si>
+  <si>
+    <t>Kundan Stones + Pearl Detailing + Emerald Green Beads + Antique Gold Finish</t>
+  </si>
+  <si>
+    <t>AD Polki + Pearl + Pink Beads + Gold Plated Finish</t>
+  </si>
+  <si>
+    <t>Antique Gold Finish + AD Stone Detailing + Filigree Work</t>
+  </si>
+  <si>
+    <t>American Diamond + Ruby Stones + Gold Plating</t>
+  </si>
+  <si>
+    <t>Ruhani</t>
+  </si>
+  <si>
+    <t>Gems &amp; Jewels</t>
+  </si>
+  <si>
+    <t>JBG-ADP-002</t>
   </si>
 </sst>
 </file>
@@ -1028,7 +1052,9 @@
   <dimension ref="A1:U6"/>
   <sheetFormatPr defaultColWidth="9.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="16384" width="9.77734375" style="1"/>
+    <col min="1" max="16" width="9.77734375" style="1"/>
+    <col min="17" max="17" width="19.5546875" style="1" customWidth="1"/>
+    <col min="18" max="16384" width="9.77734375" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
@@ -1101,7 +1127,7 @@
         <v>21</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>22</v>
@@ -1119,18 +1145,21 @@
         <v>150</v>
       </c>
       <c r="H2" s="1">
+        <f>SUM(E2:G2)</f>
         <v>625</v>
       </c>
       <c r="I2" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J2" s="1">
-        <v>3299</v>
+        <f>ROUNDUP((H2*I2)/500,0)*500-1</f>
+        <v>1999</v>
       </c>
       <c r="K2" s="1">
         <v>2</v>
       </c>
       <c r="M2" s="1">
+        <f>K2-L2</f>
         <v>2</v>
       </c>
       <c r="N2" s="1" t="s">
@@ -1140,27 +1169,27 @@
         <v>25</v>
       </c>
       <c r="Q2" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="R2" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="R2" s="1" t="s">
+      <c r="S2" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="T2" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="U2" s="1" t="s">
         <v>27</v>
-      </c>
-      <c r="S2" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="T2" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="U2" s="1" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="3" spans="1:21" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>22</v>
@@ -1178,88 +1207,233 @@
         <v>150</v>
       </c>
       <c r="H3" s="1">
+        <f>SUM(E3:G3)</f>
         <v>1415</v>
       </c>
       <c r="I3" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J3" s="1">
-        <v>3499</v>
+        <f>ROUNDUP((H3*I3)/500,0)*500-1</f>
+        <v>4499</v>
       </c>
       <c r="K3" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M3" s="1">
-        <v>2</v>
+        <f>K3-L3</f>
+        <v>1</v>
       </c>
       <c r="N3" s="1" t="s">
         <v>24</v>
       </c>
       <c r="O3" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="Q3" s="1" t="s">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="R3" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="S3" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="T3" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="U3" s="1" t="s">
         <v>27</v>
-      </c>
-      <c r="S3" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="T3" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="U3" s="1" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="4" spans="1:21" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>37</v>
+        <v>35</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>23</v>
       </c>
       <c r="E4" s="1">
         <v>1495</v>
       </c>
+      <c r="F4" s="1">
+        <v>25</v>
+      </c>
+      <c r="G4" s="1">
+        <v>150</v>
+      </c>
       <c r="H4" s="1">
-        <v>1415</v>
+        <f>SUM(E4:G4)</f>
+        <v>1670</v>
       </c>
       <c r="I4" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J4" s="1">
-        <v>3499</v>
+        <f>ROUNDUP((H4*I4)/500,0)*500-1</f>
+        <v>5499</v>
+      </c>
+      <c r="K4" s="1">
+        <v>2</v>
+      </c>
+      <c r="M4" s="1">
+        <f>K4-L4</f>
+        <v>2</v>
+      </c>
+      <c r="N4" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="O4" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q4" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="R4" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="S4" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="T4" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="U4" s="1" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="5" spans="1:21" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>38</v>
+        <v>36</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>23</v>
       </c>
       <c r="E5" s="1">
         <v>1134</v>
       </c>
+      <c r="F5" s="1">
+        <v>25</v>
+      </c>
+      <c r="G5" s="1">
+        <v>150</v>
+      </c>
       <c r="H5" s="1">
-        <v>1415</v>
+        <f>SUM(E5:G5)</f>
+        <v>1309</v>
       </c>
       <c r="I5" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J5" s="1">
-        <v>3499</v>
+        <f>ROUNDUP((H5*I5)/500,0)*500-1</f>
+        <v>3999</v>
+      </c>
+      <c r="K5" s="1">
+        <v>2</v>
+      </c>
+      <c r="M5" s="1">
+        <f>K5-L5</f>
+        <v>2</v>
+      </c>
+      <c r="N5" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="O5" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q5" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="R5" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="S5" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="T5" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="U5" s="1" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="6" spans="1:21" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>34</v>
+        <v>32</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E6" s="1">
+        <v>2100</v>
+      </c>
+      <c r="F6" s="1">
+        <v>25</v>
+      </c>
+      <c r="G6" s="1">
+        <v>150</v>
+      </c>
+      <c r="H6" s="1">
+        <f>SUM(E6:G6)</f>
+        <v>2275</v>
+      </c>
+      <c r="I6" s="1">
+        <v>1.75</v>
+      </c>
+      <c r="J6" s="1">
+        <f>ROUNDUP((H6*I6)/500,0)*500-1</f>
+        <v>3999</v>
+      </c>
+      <c r="K6" s="1">
+        <v>2</v>
+      </c>
+      <c r="M6" s="1">
+        <f>K6-L6</f>
+        <v>2</v>
+      </c>
+      <c r="N6" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="O6" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q6" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="R6" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="S6" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="T6" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="U6" s="1" t="s">
+        <v>27</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add Ruhani (₹3,999), update all prices: Kaveri 1999, Raahi 4499, Saanjh 5499, Adaa 3999
</commit_message>
<xml_diff>
--- a/business/inventory-ledger.xlsx
+++ b/business/inventory-ledger.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ahujadiv\Desktop\Team\Automations\JBG\jewels-by-geetika\business\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD8B8C02-F650-45C3-84B8-31935A18E0E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9671019-68F8-49C5-9C66-C5C70EC15859}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{68BF2D20-07EA-4E2C-B5AF-3720521CC247}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="48">
   <si>
     <t>Product ID</t>
   </si>
@@ -174,6 +174,9 @@
   </si>
   <si>
     <t>JBG-ADP-002</t>
+  </si>
+  <si>
+    <t>AD Stones + Emerald Green Beads + Silver Finish</t>
   </si>
 </sst>
 </file>
@@ -1417,7 +1420,7 @@
         <v>46</v>
       </c>
       <c r="Q6" s="1" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="R6" s="1" t="s">
         <v>26</v>

</xml_diff>

<commit_message>
Add Kanak (₹1,999), Sunehri (₹999), Virasat (₹999) - rings category
</commit_message>
<xml_diff>
--- a/business/inventory-ledger.xlsx
+++ b/business/inventory-ledger.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ahujadiv\Desktop\Team\Automations\JBG\jewels-by-geetika\business\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9671019-68F8-49C5-9C66-C5C70EC15859}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E68EA08-9BEC-49AF-B0C4-DB7361983089}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{68BF2D20-07EA-4E2C-B5AF-3720521CC247}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="57">
   <si>
     <t>Product ID</t>
   </si>
@@ -177,6 +177,33 @@
   </si>
   <si>
     <t>AD Stones + Emerald Green Beads + Silver Finish</t>
+  </si>
+  <si>
+    <t>Kanak</t>
+  </si>
+  <si>
+    <t>Antique Gold Finish + Filigree Detailing + Premium Stone Accents</t>
+  </si>
+  <si>
+    <t>JBG-006</t>
+  </si>
+  <si>
+    <t>JBG-NCK-004</t>
+  </si>
+  <si>
+    <t>Virasat</t>
+  </si>
+  <si>
+    <t>JBG-007</t>
+  </si>
+  <si>
+    <t>Ring</t>
+  </si>
+  <si>
+    <t>JBG-RNG-001</t>
+  </si>
+  <si>
+    <t>Antique Gold Finish + Peacock Motif Detailing + Emerald Enamel Accents + Premium Stone Embellishments + Ghungroo Danglings</t>
   </si>
 </sst>
 </file>
@@ -1052,7 +1079,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{39C98BD1-4979-45B2-A4A1-1CB48783F5EE}">
-  <dimension ref="A1:U6"/>
+  <dimension ref="A1:U8"/>
   <sheetFormatPr defaultColWidth="9.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="16" width="9.77734375" style="1"/>
@@ -1435,6 +1462,129 @@
         <v>27</v>
       </c>
     </row>
+    <row r="7" spans="1:21" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E7" s="1">
+        <v>472</v>
+      </c>
+      <c r="F7" s="1">
+        <v>30</v>
+      </c>
+      <c r="G7" s="1">
+        <v>150</v>
+      </c>
+      <c r="H7" s="1">
+        <f>SUM(E7:G7)</f>
+        <v>652</v>
+      </c>
+      <c r="I7" s="1">
+        <v>3</v>
+      </c>
+      <c r="J7" s="1">
+        <f>ROUNDUP((H7*I7)/500,0)*500-1</f>
+        <v>1999</v>
+      </c>
+      <c r="K7" s="1">
+        <v>2</v>
+      </c>
+      <c r="M7" s="1">
+        <f>K7-L7</f>
+        <v>2</v>
+      </c>
+      <c r="N7" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="O7" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="Q7" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="R7" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="S7" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="T7" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="U7" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="8" spans="1:21" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E8" s="1">
+        <v>71</v>
+      </c>
+      <c r="F8" s="1">
+        <v>30</v>
+      </c>
+      <c r="G8" s="1">
+        <v>150</v>
+      </c>
+      <c r="H8" s="1">
+        <f>SUM(E8:G8)</f>
+        <v>251</v>
+      </c>
+      <c r="I8" s="1">
+        <v>3</v>
+      </c>
+      <c r="J8" s="1">
+        <f>ROUNDUP((H8*I8)/500,0)*500-1</f>
+        <v>999</v>
+      </c>
+      <c r="K8" s="1">
+        <v>1</v>
+      </c>
+      <c r="M8" s="1">
+        <v>1</v>
+      </c>
+      <c r="N8" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="O8" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="Q8" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="R8" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="S8" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="T8" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="U8" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Fix stats label, confirm real images in Brand Story and Instagram sections
</commit_message>
<xml_diff>
--- a/business/inventory-ledger.xlsx
+++ b/business/inventory-ledger.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ahujadiv\Desktop\Team\Automations\JBG\jewels-by-geetika\business\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E68EA08-9BEC-49AF-B0C4-DB7361983089}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B847AFA-2907-4E2C-8202-D9D05C792B29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{68BF2D20-07EA-4E2C-B5AF-3720521CC247}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="74">
   <si>
     <t>Product ID</t>
   </si>
@@ -80,9 +80,6 @@
     <t>SKU</t>
   </si>
   <si>
-    <t>Weight (g)</t>
-  </si>
-  <si>
     <t>Material</t>
   </si>
   <si>
@@ -204,6 +201,60 @@
   </si>
   <si>
     <t>Antique Gold Finish + Peacock Motif Detailing + Emerald Enamel Accents + Premium Stone Embellishments + Ghungroo Danglings</t>
+  </si>
+  <si>
+    <t>Antique Gold Finish + Kundan Stones + Ruby &amp; Emerald Tone Stones + Ghungroo Charms + Adjustable Ring Base</t>
+  </si>
+  <si>
+    <t>JBG-008</t>
+  </si>
+  <si>
+    <t>Sunehri</t>
+  </si>
+  <si>
+    <t>JBG-RNG-002</t>
+  </si>
+  <si>
+    <t>Antara</t>
+  </si>
+  <si>
+    <t>JBG-009</t>
+  </si>
+  <si>
+    <t>Antique Gold Finish + Temple Motif Detailing + Premium CZ Stones + Pearl Danglings + Green Bead Accents</t>
+  </si>
+  <si>
+    <t>Temple Jewellery</t>
+  </si>
+  <si>
+    <t>JBG-TMJ-001</t>
+  </si>
+  <si>
+    <t>JBG-010</t>
+  </si>
+  <si>
+    <t>Chandni</t>
+  </si>
+  <si>
+    <t>JBG-011</t>
+  </si>
+  <si>
+    <t>Rajsi</t>
+  </si>
+  <si>
+    <t>American Diamond + Emerald Green Stone + Premium Gold Finish + Intricate Zircon Detailing</t>
+  </si>
+  <si>
+    <t>JBG-ADP-003</t>
+  </si>
+  <si>
+    <t>AD Stones + Emerald Green Stone Accents + Pearl Danglings + Antique Gold Finish</t>
+  </si>
+  <si>
+    <t>AD - Necklace</t>
+  </si>
+  <si>
+    <t>JBG-ADN-001</t>
   </si>
 </sst>
 </file>
@@ -1079,15 +1130,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{39C98BD1-4979-45B2-A4A1-1CB48783F5EE}">
-  <dimension ref="A1:U8"/>
+  <dimension ref="A1:T56"/>
   <sheetFormatPr defaultColWidth="9.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="16" width="9.77734375" style="1"/>
-    <col min="17" max="17" width="19.5546875" style="1" customWidth="1"/>
-    <col min="18" max="16384" width="9.77734375" style="1"/>
+    <col min="1" max="15" width="9.77734375" style="1"/>
+    <col min="16" max="16" width="19.5546875" style="1" customWidth="1"/>
+    <col min="17" max="16384" width="9.77734375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:20" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1148,413 +1199,410 @@
       <c r="T1" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="2" t="s">
+    </row>
+    <row r="2" spans="1:20" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="2" spans="1:21" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
+      <c r="B2" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B2" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="C2" s="1" t="s">
+      <c r="D2" s="1" t="s">
         <v>22</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>23</v>
       </c>
       <c r="E2" s="1">
         <v>450</v>
       </c>
       <c r="F2" s="1">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="G2" s="1">
         <v>150</v>
       </c>
       <c r="H2" s="1">
-        <f>SUM(E2:G2)</f>
-        <v>625</v>
+        <f t="shared" ref="H2:H12" si="0">SUM(E2:G2)</f>
+        <v>650</v>
       </c>
       <c r="I2" s="1">
         <v>3</v>
       </c>
       <c r="J2" s="1">
-        <f>ROUNDUP((H2*I2)/500,0)*500-1</f>
+        <f t="shared" ref="J2:J12" si="1">ROUNDUP((H2*I2)/500,0)*500-1</f>
         <v>1999</v>
       </c>
       <c r="K2" s="1">
         <v>2</v>
       </c>
       <c r="M2" s="1">
-        <f>K2-L2</f>
+        <f t="shared" ref="M2:M7" si="2">K2-L2</f>
         <v>2</v>
       </c>
       <c r="N2" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="O2" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="O2" s="1" t="s">
-        <v>25</v>
+      <c r="P2" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="Q2" s="1" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
       <c r="R2" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="S2" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="T2" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="U2" s="1" t="s">
+    </row>
+    <row r="3" spans="1:20" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="3" spans="1:21" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
-        <v>28</v>
-      </c>
       <c r="B3" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C3" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D3" s="1" t="s">
         <v>22</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>23</v>
       </c>
       <c r="E3" s="1">
         <v>1240</v>
       </c>
       <c r="F3" s="1">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="G3" s="1">
         <v>150</v>
       </c>
       <c r="H3" s="1">
-        <f>SUM(E3:G3)</f>
-        <v>1415</v>
+        <f t="shared" si="0"/>
+        <v>1440</v>
       </c>
       <c r="I3" s="1">
         <v>3</v>
       </c>
       <c r="J3" s="1">
-        <f>ROUNDUP((H3*I3)/500,0)*500-1</f>
+        <f t="shared" si="1"/>
         <v>4499</v>
       </c>
       <c r="K3" s="1">
         <v>1</v>
       </c>
       <c r="M3" s="1">
-        <f>K3-L3</f>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="N3" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="O3" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
+      </c>
+      <c r="P3" s="1" t="s">
+        <v>40</v>
       </c>
       <c r="Q3" s="1" t="s">
-        <v>41</v>
+        <v>25</v>
       </c>
       <c r="R3" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="S3" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="T3" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="U3" s="1" t="s">
-        <v>27</v>
-      </c>
     </row>
-    <row r="4" spans="1:21" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:20" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C4" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D4" s="1" t="s">
         <v>22</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>23</v>
       </c>
       <c r="E4" s="1">
         <v>1495</v>
       </c>
       <c r="F4" s="1">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="G4" s="1">
         <v>150</v>
       </c>
       <c r="H4" s="1">
-        <f>SUM(E4:G4)</f>
-        <v>1670</v>
+        <f t="shared" si="0"/>
+        <v>1695</v>
       </c>
       <c r="I4" s="1">
         <v>3</v>
       </c>
       <c r="J4" s="1">
-        <f>ROUNDUP((H4*I4)/500,0)*500-1</f>
+        <f t="shared" si="1"/>
         <v>5499</v>
       </c>
       <c r="K4" s="1">
         <v>2</v>
       </c>
       <c r="M4" s="1">
-        <f>K4-L4</f>
+        <f t="shared" si="2"/>
         <v>2</v>
       </c>
       <c r="N4" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="O4" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
+      </c>
+      <c r="P4" s="1" t="s">
+        <v>39</v>
       </c>
       <c r="Q4" s="1" t="s">
-        <v>40</v>
+        <v>25</v>
       </c>
       <c r="R4" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="S4" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="T4" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="U4" s="1" t="s">
-        <v>27</v>
-      </c>
     </row>
-    <row r="5" spans="1:21" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:20" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B5" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="C5" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="C5" s="1" t="s">
-        <v>37</v>
-      </c>
       <c r="D5" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E5" s="1">
         <v>1134</v>
       </c>
       <c r="F5" s="1">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="G5" s="1">
         <v>150</v>
       </c>
       <c r="H5" s="1">
-        <f>SUM(E5:G5)</f>
-        <v>1309</v>
+        <f t="shared" si="0"/>
+        <v>1314</v>
       </c>
       <c r="I5" s="1">
         <v>3</v>
       </c>
       <c r="J5" s="1">
-        <f>ROUNDUP((H5*I5)/500,0)*500-1</f>
+        <f t="shared" si="1"/>
         <v>3999</v>
       </c>
       <c r="K5" s="1">
         <v>2</v>
       </c>
       <c r="M5" s="1">
-        <f>K5-L5</f>
+        <f t="shared" si="2"/>
         <v>2</v>
       </c>
       <c r="N5" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="O5" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
+      </c>
+      <c r="P5" s="1" t="s">
+        <v>42</v>
       </c>
       <c r="Q5" s="1" t="s">
-        <v>43</v>
+        <v>25</v>
       </c>
       <c r="R5" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="S5" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="T5" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="U5" s="1" t="s">
-        <v>27</v>
-      </c>
     </row>
-    <row r="6" spans="1:21" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:20" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B6" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="D6" s="1" t="s">
         <v>44</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>45</v>
       </c>
       <c r="E6" s="1">
         <v>2100</v>
       </c>
       <c r="F6" s="1">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="G6" s="1">
         <v>150</v>
       </c>
       <c r="H6" s="1">
-        <f>SUM(E6:G6)</f>
-        <v>2275</v>
+        <f t="shared" si="0"/>
+        <v>2280</v>
       </c>
       <c r="I6" s="1">
         <v>1.75</v>
       </c>
       <c r="J6" s="1">
-        <f>ROUNDUP((H6*I6)/500,0)*500-1</f>
+        <f t="shared" si="1"/>
         <v>3999</v>
       </c>
       <c r="K6" s="1">
         <v>2</v>
       </c>
       <c r="M6" s="1">
-        <f>K6-L6</f>
+        <f t="shared" si="2"/>
         <v>2</v>
       </c>
       <c r="N6" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="O6" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="P6" s="1" t="s">
         <v>46</v>
       </c>
       <c r="Q6" s="1" t="s">
-        <v>47</v>
+        <v>25</v>
       </c>
       <c r="R6" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="S6" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="T6" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="U6" s="1" t="s">
-        <v>27</v>
-      </c>
     </row>
-    <row r="7" spans="1:21" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:20" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C7" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D7" s="1" t="s">
         <v>22</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>23</v>
       </c>
       <c r="E7" s="1">
         <v>472</v>
       </c>
       <c r="F7" s="1">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="G7" s="1">
         <v>150</v>
       </c>
       <c r="H7" s="1">
-        <f>SUM(E7:G7)</f>
-        <v>652</v>
+        <f t="shared" si="0"/>
+        <v>672</v>
       </c>
       <c r="I7" s="1">
         <v>3</v>
       </c>
       <c r="J7" s="1">
-        <f>ROUNDUP((H7*I7)/500,0)*500-1</f>
-        <v>1999</v>
+        <f t="shared" si="1"/>
+        <v>2499</v>
       </c>
       <c r="K7" s="1">
         <v>2</v>
       </c>
       <c r="M7" s="1">
-        <f>K7-L7</f>
+        <f t="shared" si="2"/>
         <v>2</v>
       </c>
       <c r="N7" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="O7" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
+      </c>
+      <c r="P7" s="1" t="s">
+        <v>48</v>
       </c>
       <c r="Q7" s="1" t="s">
-        <v>49</v>
+        <v>25</v>
       </c>
       <c r="R7" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="S7" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="T7" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="U7" s="1" t="s">
-        <v>27</v>
-      </c>
     </row>
-    <row r="8" spans="1:21" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:20" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C8" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="B8" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>54</v>
-      </c>
       <c r="D8" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E8" s="1">
         <v>71</v>
       </c>
       <c r="F8" s="1">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="G8" s="1">
         <v>150</v>
       </c>
       <c r="H8" s="1">
-        <f>SUM(E8:G8)</f>
-        <v>251</v>
+        <f t="shared" si="0"/>
+        <v>271</v>
       </c>
       <c r="I8" s="1">
         <v>3</v>
       </c>
       <c r="J8" s="1">
-        <f>ROUNDUP((H8*I8)/500,0)*500-1</f>
+        <f t="shared" si="1"/>
         <v>999</v>
       </c>
       <c r="K8" s="1">
@@ -1564,27 +1612,315 @@
         <v>1</v>
       </c>
       <c r="N8" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="O8" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="P8" s="1" t="s">
         <v>55</v>
       </c>
       <c r="Q8" s="1" t="s">
-        <v>56</v>
+        <v>25</v>
       </c>
       <c r="R8" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="S8" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="T8" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="U8" s="1" t="s">
-        <v>27</v>
-      </c>
     </row>
+    <row r="9" spans="1:20" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E9" s="1">
+        <v>110</v>
+      </c>
+      <c r="F9" s="1">
+        <v>50</v>
+      </c>
+      <c r="G9" s="1">
+        <v>150</v>
+      </c>
+      <c r="H9" s="1">
+        <f t="shared" si="0"/>
+        <v>310</v>
+      </c>
+      <c r="I9" s="1">
+        <v>3</v>
+      </c>
+      <c r="J9" s="1">
+        <f t="shared" si="1"/>
+        <v>999</v>
+      </c>
+      <c r="K9" s="1">
+        <v>2</v>
+      </c>
+      <c r="M9" s="1">
+        <v>2</v>
+      </c>
+      <c r="N9" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="O9" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="P9" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="Q9" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="R9" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="S9" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="T9" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="10" spans="1:20" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E10" s="1">
+        <v>1070</v>
+      </c>
+      <c r="F10" s="1">
+        <v>50</v>
+      </c>
+      <c r="G10" s="1">
+        <v>150</v>
+      </c>
+      <c r="H10" s="1">
+        <f t="shared" si="0"/>
+        <v>1270</v>
+      </c>
+      <c r="I10" s="1">
+        <v>3</v>
+      </c>
+      <c r="J10" s="1">
+        <f t="shared" si="1"/>
+        <v>3999</v>
+      </c>
+      <c r="K10" s="1">
+        <v>2</v>
+      </c>
+      <c r="M10" s="1">
+        <v>2</v>
+      </c>
+      <c r="N10" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="O10" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="P10" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="Q10" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="R10" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="S10" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="T10" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="11" spans="1:20" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E11" s="1">
+        <v>1069</v>
+      </c>
+      <c r="F11" s="1">
+        <v>50</v>
+      </c>
+      <c r="G11" s="1">
+        <v>150</v>
+      </c>
+      <c r="H11" s="1">
+        <f t="shared" si="0"/>
+        <v>1269</v>
+      </c>
+      <c r="I11" s="1">
+        <v>3</v>
+      </c>
+      <c r="J11" s="1">
+        <f t="shared" si="1"/>
+        <v>3999</v>
+      </c>
+      <c r="K11" s="1">
+        <v>2</v>
+      </c>
+      <c r="M11" s="1">
+        <v>2</v>
+      </c>
+      <c r="N11" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="O11" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="P11" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="Q11" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="R11" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="S11" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="T11" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="12" spans="1:20" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E12" s="1">
+        <v>654</v>
+      </c>
+      <c r="F12" s="1">
+        <v>50</v>
+      </c>
+      <c r="G12" s="1">
+        <v>150</v>
+      </c>
+      <c r="H12" s="1">
+        <f t="shared" si="0"/>
+        <v>854</v>
+      </c>
+      <c r="I12" s="1">
+        <v>3</v>
+      </c>
+      <c r="J12" s="1">
+        <f t="shared" si="1"/>
+        <v>2999</v>
+      </c>
+      <c r="K12" s="1">
+        <v>2</v>
+      </c>
+      <c r="M12" s="1">
+        <v>2</v>
+      </c>
+      <c r="N12" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="O12" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="P12" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="Q12" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="R12" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="S12" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="T12" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="13" spans="1:20" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="14" spans="1:20" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="15" spans="1:20" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="16" spans="1:20" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="17" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="18" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="19" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="20" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="21" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="22" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="23" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="24" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="25" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="26" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="27" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="28" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="29" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="30" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="31" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="32" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="33" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="34" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="35" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="36" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="37" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="38" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="39" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="40" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="41" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="42" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="43" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="44" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="45" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="46" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="47" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="48" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="49" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="50" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="51" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="52" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="53" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="54" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="55" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="56" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Add 5 new products (Bella, Blossom, Ziya, Grace, Iris), Earrings + Anti Tarnish categories
</commit_message>
<xml_diff>
--- a/business/inventory-ledger.xlsx
+++ b/business/inventory-ledger.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ahujadiv\Desktop\Team\Automations\JBG\jewels-by-geetika\business\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B847AFA-2907-4E2C-8202-D9D05C792B29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{444EC0F0-1DAE-448A-8095-CBF5D85B17D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{68BF2D20-07EA-4E2C-B5AF-3720521CC247}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="92">
   <si>
     <t>Product ID</t>
   </si>
@@ -255,6 +255,60 @@
   </si>
   <si>
     <t>JBG-ADN-001</t>
+  </si>
+  <si>
+    <t>JBG-012</t>
+  </si>
+  <si>
+    <t>Bella</t>
+  </si>
+  <si>
+    <t>AT-Necklace</t>
+  </si>
+  <si>
+    <t>Blossom</t>
+  </si>
+  <si>
+    <t>Ziya</t>
+  </si>
+  <si>
+    <t>Iris</t>
+  </si>
+  <si>
+    <t>Grace</t>
+  </si>
+  <si>
+    <t>AT-Earrings</t>
+  </si>
+  <si>
+    <t>JBG-ATN-001</t>
+  </si>
+  <si>
+    <t>JBG-ATE-001</t>
+  </si>
+  <si>
+    <t>JBG-ATN-002</t>
+  </si>
+  <si>
+    <t>JBG-ATE-002</t>
+  </si>
+  <si>
+    <t>JBG-ATE-003</t>
+  </si>
+  <si>
+    <t>Cubic Zirconia + Stainless Steel + Gold Plating</t>
+  </si>
+  <si>
+    <t>Premium Anti Tarnish Finish + Sculpted Floral Pendant + Gold Tone Snake Chain</t>
+  </si>
+  <si>
+    <t>Gold Finish Floral Metal + Premium Crystal Stones + Pearl Drop</t>
+  </si>
+  <si>
+    <t>Pearl + Blush Crystal Stones + Gold Finish + Pearl Drops</t>
+  </si>
+  <si>
+    <t>Gold Finish + Blue Evil Eye Stone + Crystal Embellishments + Sculpted Metal Detailing</t>
   </si>
 </sst>
 </file>
@@ -1877,26 +1931,330 @@
         <v>26</v>
       </c>
     </row>
-    <row r="13" spans="1:20" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="14" spans="1:20" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="15" spans="1:20" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="16" spans="1:20" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="17" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="18" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="19" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="20" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="21" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="22" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="23" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="24" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="25" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="26" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="27" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="28" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="29" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="30" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="31" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="32" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="13" spans="1:20" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E13" s="1">
+        <v>456</v>
+      </c>
+      <c r="F13" s="1">
+        <v>50</v>
+      </c>
+      <c r="G13" s="1">
+        <v>150</v>
+      </c>
+      <c r="H13" s="1">
+        <f t="shared" ref="H13" si="3">SUM(E13:G13)</f>
+        <v>656</v>
+      </c>
+      <c r="I13" s="1">
+        <v>3</v>
+      </c>
+      <c r="J13" s="1">
+        <f t="shared" ref="J13" si="4">ROUNDUP((H13*I13)/500,0)*500-1</f>
+        <v>1999</v>
+      </c>
+      <c r="K13" s="1">
+        <v>2</v>
+      </c>
+      <c r="M13" s="1">
+        <v>2</v>
+      </c>
+      <c r="N13" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="O13" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="P13" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="Q13" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="R13" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="S13" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="T13" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="14" spans="1:20" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="1" t="str">
+        <f>LEFT(A13,4)&amp;TEXT(RIGHT(A13,3)+1,"000")</f>
+        <v>JBG-013</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E14" s="1">
+        <v>145</v>
+      </c>
+      <c r="F14" s="1">
+        <v>50</v>
+      </c>
+      <c r="G14" s="1">
+        <v>150</v>
+      </c>
+      <c r="H14" s="1">
+        <f t="shared" ref="H14:H17" si="5">SUM(E14:G14)</f>
+        <v>345</v>
+      </c>
+      <c r="I14" s="1">
+        <v>3</v>
+      </c>
+      <c r="J14" s="1">
+        <f t="shared" ref="J14:J17" si="6">ROUNDUP((H14*I14)/500,0)*500-1</f>
+        <v>1499</v>
+      </c>
+      <c r="K14" s="1">
+        <v>2</v>
+      </c>
+      <c r="M14" s="1">
+        <v>2</v>
+      </c>
+      <c r="N14" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="O14" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="P14" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="Q14" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="R14" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="S14" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="T14" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="15" spans="1:20" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="1" t="str">
+        <f>LEFT(A14,4)&amp;TEXT(RIGHT(A14,3)+1,"000")</f>
+        <v>JBG-014</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E15" s="1">
+        <v>380</v>
+      </c>
+      <c r="F15" s="1">
+        <v>50</v>
+      </c>
+      <c r="G15" s="1">
+        <v>150</v>
+      </c>
+      <c r="H15" s="1">
+        <f t="shared" si="5"/>
+        <v>580</v>
+      </c>
+      <c r="I15" s="1">
+        <v>2.5</v>
+      </c>
+      <c r="J15" s="1">
+        <f t="shared" si="6"/>
+        <v>1499</v>
+      </c>
+      <c r="K15" s="1">
+        <v>2</v>
+      </c>
+      <c r="M15" s="1">
+        <v>2</v>
+      </c>
+      <c r="N15" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="O15" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="P15" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="Q15" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="R15" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="S15" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="T15" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="16" spans="1:20" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="1" t="str">
+        <f>LEFT(A15,4)&amp;TEXT(RIGHT(A15,3)+1,"000")</f>
+        <v>JBG-015</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E16" s="1">
+        <v>480</v>
+      </c>
+      <c r="F16" s="1">
+        <v>50</v>
+      </c>
+      <c r="G16" s="1">
+        <v>150</v>
+      </c>
+      <c r="H16" s="1">
+        <f t="shared" si="5"/>
+        <v>680</v>
+      </c>
+      <c r="I16" s="1">
+        <v>2.5</v>
+      </c>
+      <c r="J16" s="1">
+        <f t="shared" si="6"/>
+        <v>1999</v>
+      </c>
+      <c r="K16" s="1">
+        <v>2</v>
+      </c>
+      <c r="M16" s="1">
+        <v>2</v>
+      </c>
+      <c r="N16" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="O16" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="P16" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="Q16" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="R16" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="S16" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="T16" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="17" spans="1:20" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="1" t="str">
+        <f>LEFT(A16,4)&amp;TEXT(RIGHT(A16,3)+1,"000")</f>
+        <v>JBG-016</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E17" s="1">
+        <v>425</v>
+      </c>
+      <c r="F17" s="1">
+        <v>50</v>
+      </c>
+      <c r="G17" s="1">
+        <v>150</v>
+      </c>
+      <c r="H17" s="1">
+        <f t="shared" si="5"/>
+        <v>625</v>
+      </c>
+      <c r="I17" s="1">
+        <v>2</v>
+      </c>
+      <c r="J17" s="1">
+        <f t="shared" si="6"/>
+        <v>1499</v>
+      </c>
+      <c r="K17" s="1">
+        <v>1</v>
+      </c>
+      <c r="M17" s="1">
+        <v>1</v>
+      </c>
+      <c r="N17" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="O17" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="P17" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="Q17" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="R17" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="S17" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="T17" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="18" spans="1:20" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="19" spans="1:20" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="20" spans="1:20" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="21" spans="1:20" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="22" spans="1:20" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="23" spans="1:20" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="24" spans="1:20" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="25" spans="1:20" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="26" spans="1:20" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="27" spans="1:20" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="28" spans="1:20" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="29" spans="1:20" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="30" spans="1:20" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="31" spans="1:20" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="32" spans="1:20" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="33" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="34" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="35" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
@@ -1924,5 +2282,8 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <ignoredErrors>
+    <ignoredError sqref="H13" formula="1"/>
+  </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 7 new products (Stella, Hope, Luna, Lily, Daisy, Zahara) + Bracelets category
</commit_message>
<xml_diff>
--- a/business/inventory-ledger.xlsx
+++ b/business/inventory-ledger.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ahujadiv\Desktop\Team\Automations\JBG\jewels-by-geetika\business\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{444EC0F0-1DAE-448A-8095-CBF5D85B17D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A717F24C-CD11-42E0-858F-2747C58DCD80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{68BF2D20-07EA-4E2C-B5AF-3720521CC247}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="82">
   <si>
     <t>Product ID</t>
   </si>
@@ -80,21 +80,6 @@
     <t>SKU</t>
   </si>
   <si>
-    <t>Material</t>
-  </si>
-  <si>
-    <t>Images Uploaded</t>
-  </si>
-  <si>
-    <t>Listed on Website</t>
-  </si>
-  <si>
-    <t>Listed on Instagram</t>
-  </si>
-  <si>
-    <t>Notes</t>
-  </si>
-  <si>
     <t>JBG-001</t>
   </si>
   <si>
@@ -110,12 +95,6 @@
     <t>JBG-NCK-001</t>
   </si>
   <si>
-    <t>Yes</t>
-  </si>
-  <si>
-    <t>New Launch</t>
-  </si>
-  <si>
     <t>JBG-002</t>
   </si>
   <si>
@@ -152,18 +131,6 @@
     <t>JBG-ADP-001</t>
   </si>
   <si>
-    <t>Kundan Stones + Pearl Detailing + Emerald Green Beads + Antique Gold Finish</t>
-  </si>
-  <si>
-    <t>AD Polki + Pearl + Pink Beads + Gold Plated Finish</t>
-  </si>
-  <si>
-    <t>Antique Gold Finish + AD Stone Detailing + Filigree Work</t>
-  </si>
-  <si>
-    <t>American Diamond + Ruby Stones + Gold Plating</t>
-  </si>
-  <si>
     <t>Ruhani</t>
   </si>
   <si>
@@ -173,15 +140,9 @@
     <t>JBG-ADP-002</t>
   </si>
   <si>
-    <t>AD Stones + Emerald Green Beads + Silver Finish</t>
-  </si>
-  <si>
     <t>Kanak</t>
   </si>
   <si>
-    <t>Antique Gold Finish + Filigree Detailing + Premium Stone Accents</t>
-  </si>
-  <si>
     <t>JBG-006</t>
   </si>
   <si>
@@ -200,12 +161,6 @@
     <t>JBG-RNG-001</t>
   </si>
   <si>
-    <t>Antique Gold Finish + Peacock Motif Detailing + Emerald Enamel Accents + Premium Stone Embellishments + Ghungroo Danglings</t>
-  </si>
-  <si>
-    <t>Antique Gold Finish + Kundan Stones + Ruby &amp; Emerald Tone Stones + Ghungroo Charms + Adjustable Ring Base</t>
-  </si>
-  <si>
     <t>JBG-008</t>
   </si>
   <si>
@@ -221,9 +176,6 @@
     <t>JBG-009</t>
   </si>
   <si>
-    <t>Antique Gold Finish + Temple Motif Detailing + Premium CZ Stones + Pearl Danglings + Green Bead Accents</t>
-  </si>
-  <si>
     <t>Temple Jewellery</t>
   </si>
   <si>
@@ -242,15 +194,9 @@
     <t>Rajsi</t>
   </si>
   <si>
-    <t>American Diamond + Emerald Green Stone + Premium Gold Finish + Intricate Zircon Detailing</t>
-  </si>
-  <si>
     <t>JBG-ADP-003</t>
   </si>
   <si>
-    <t>AD Stones + Emerald Green Stone Accents + Pearl Danglings + Antique Gold Finish</t>
-  </si>
-  <si>
     <t>AD - Necklace</t>
   </si>
   <si>
@@ -296,26 +242,50 @@
     <t>JBG-ATE-003</t>
   </si>
   <si>
-    <t>Cubic Zirconia + Stainless Steel + Gold Plating</t>
-  </si>
-  <si>
-    <t>Premium Anti Tarnish Finish + Sculpted Floral Pendant + Gold Tone Snake Chain</t>
-  </si>
-  <si>
-    <t>Gold Finish Floral Metal + Premium Crystal Stones + Pearl Drop</t>
-  </si>
-  <si>
-    <t>Pearl + Blush Crystal Stones + Gold Finish + Pearl Drops</t>
-  </si>
-  <si>
-    <t>Gold Finish + Blue Evil Eye Stone + Crystal Embellishments + Sculpted Metal Detailing</t>
+    <t>Golden Lobster</t>
+  </si>
+  <si>
+    <t>JBG-ATN-003</t>
+  </si>
+  <si>
+    <t>Hope</t>
+  </si>
+  <si>
+    <t>Luna</t>
+  </si>
+  <si>
+    <t>JBG-ATN-004</t>
+  </si>
+  <si>
+    <t>Lily</t>
+  </si>
+  <si>
+    <t>JBG-ATN-005</t>
+  </si>
+  <si>
+    <t>JBG-ATN-006</t>
+  </si>
+  <si>
+    <t>Daisy</t>
+  </si>
+  <si>
+    <t>Zahara</t>
+  </si>
+  <si>
+    <t>AT-Bracelet</t>
+  </si>
+  <si>
+    <t>JBG-ATB-001</t>
+  </si>
+  <si>
+    <t>JBG-ATB-002</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -446,6 +416,12 @@
     <font>
       <sz val="11"/>
       <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -798,7 +774,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -808,6 +784,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="0" xfId="7" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="4" borderId="0" xfId="8" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="42">
@@ -854,7 +836,18 @@
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
     <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="1">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -1184,15 +1177,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{39C98BD1-4979-45B2-A4A1-1CB48783F5EE}">
-  <dimension ref="A1:T56"/>
+  <dimension ref="A1:O56"/>
   <sheetFormatPr defaultColWidth="9.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="15" width="9.77734375" style="1"/>
-    <col min="16" max="16" width="19.5546875" style="1" customWidth="1"/>
-    <col min="17" max="16384" width="9.77734375" style="1"/>
+    <col min="1" max="16384" width="9.77734375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:15" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1238,34 +1229,19 @@
       <c r="O1" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="2" t="s">
+    </row>
+    <row r="2" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="2" t="s">
+      <c r="B2" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="2" t="s">
+      <c r="D2" s="1" t="s">
         <v>17</v>
-      </c>
-      <c r="S1" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="T1" s="2" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="2" spans="1:20" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>22</v>
       </c>
       <c r="E2" s="1">
         <v>450</v>
@@ -1291,43 +1267,28 @@
         <v>2</v>
       </c>
       <c r="M2" s="1">
-        <f t="shared" ref="M2:M7" si="2">K2-L2</f>
+        <f>K2-L2</f>
         <v>2</v>
       </c>
       <c r="N2" s="1" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="O2" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="P2" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="Q2" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="R2" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="S2" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="T2" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="3" spans="1:20" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>33</v>
-      </c>
       <c r="C3" s="1" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="E3" s="1">
         <v>1240</v>
@@ -1353,43 +1314,28 @@
         <v>1</v>
       </c>
       <c r="M3" s="1">
-        <f t="shared" si="2"/>
+        <f t="shared" ref="M3:M17" si="2">K3-L3</f>
         <v>1</v>
       </c>
       <c r="N3" s="1" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="O3" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="P3" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="Q3" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="R3" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="S3" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="T3" s="1" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:20" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="E4" s="1">
         <v>1495</v>
@@ -1419,39 +1365,24 @@
         <v>2</v>
       </c>
       <c r="N4" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="O4" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="O4" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="P4" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="Q4" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="R4" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="S4" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="T4" s="1" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="5" spans="1:20" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="1" t="s">
-        <v>30</v>
-      </c>
       <c r="B5" s="3" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="E5" s="1">
         <v>1134</v>
@@ -1481,39 +1412,24 @@
         <v>2</v>
       </c>
       <c r="N5" s="1" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="O5" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="P5" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="Q5" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="R5" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="S5" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="T5" s="1" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
     </row>
-    <row r="6" spans="1:20" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>44</v>
+        <v>33</v>
       </c>
       <c r="E6" s="1">
         <v>2100</v>
@@ -1543,39 +1459,24 @@
         <v>2</v>
       </c>
       <c r="N6" s="1" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="O6" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="P6" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="Q6" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="R6" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="S6" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="T6" s="1" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
     </row>
-    <row r="7" spans="1:20" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>49</v>
+        <v>36</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>47</v>
+        <v>35</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="E7" s="1">
         <v>472</v>
@@ -1605,100 +1506,74 @@
         <v>2</v>
       </c>
       <c r="N7" s="1" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="O7" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E8" s="4">
+        <v>71</v>
+      </c>
+      <c r="F8" s="4">
         <v>50</v>
       </c>
-      <c r="P7" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="Q7" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="R7" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="S7" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="T7" s="1" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="8" spans="1:20" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="E8" s="1">
-        <v>71</v>
-      </c>
-      <c r="F8" s="1">
-        <v>50</v>
-      </c>
-      <c r="G8" s="1">
+      <c r="G8" s="4">
         <v>150</v>
       </c>
-      <c r="H8" s="1">
+      <c r="H8" s="4">
         <f t="shared" si="0"/>
         <v>271</v>
       </c>
-      <c r="I8" s="1">
+      <c r="I8" s="4">
         <v>3</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="4">
         <f t="shared" si="1"/>
         <v>999</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="4">
         <v>1</v>
       </c>
-      <c r="M8" s="1">
+      <c r="L8" s="4">
         <v>1</v>
       </c>
-      <c r="N8" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="O8" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="P8" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="Q8" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="R8" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="S8" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="T8" s="1" t="s">
-        <v>26</v>
+      <c r="M8" s="4">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="N8" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="O8" s="4" t="s">
+        <v>41</v>
       </c>
     </row>
-    <row r="9" spans="1:20" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
-        <v>57</v>
+        <v>42</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>58</v>
+        <v>43</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>53</v>
+        <v>40</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="E9" s="1">
         <v>110</v>
@@ -1724,42 +1599,28 @@
         <v>2</v>
       </c>
       <c r="M9" s="1">
+        <f t="shared" si="2"/>
         <v>2</v>
       </c>
       <c r="N9" s="1" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="O9" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="P9" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="Q9" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="R9" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="S9" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="T9" s="1" t="s">
-        <v>26</v>
+        <v>44</v>
       </c>
     </row>
-    <row r="10" spans="1:20" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
-        <v>61</v>
+        <v>46</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>60</v>
+        <v>45</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="E10" s="1">
         <v>1070</v>
@@ -1785,42 +1646,28 @@
         <v>2</v>
       </c>
       <c r="M10" s="1">
+        <f t="shared" si="2"/>
         <v>2</v>
       </c>
       <c r="N10" s="1" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="O10" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="P10" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="Q10" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="R10" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="S10" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="T10" s="1" t="s">
-        <v>26</v>
+        <v>48</v>
       </c>
     </row>
-    <row r="11" spans="1:20" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
-        <v>65</v>
+        <v>49</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>66</v>
+        <v>50</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="E11" s="1">
         <v>1069</v>
@@ -1846,42 +1693,28 @@
         <v>2</v>
       </c>
       <c r="M11" s="1">
+        <f t="shared" si="2"/>
         <v>2</v>
       </c>
       <c r="N11" s="1" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="O11" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="P11" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="Q11" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="R11" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="S11" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="T11" s="1" t="s">
-        <v>26</v>
+        <v>53</v>
       </c>
     </row>
-    <row r="12" spans="1:20" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
-        <v>67</v>
+        <v>51</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>68</v>
+        <v>52</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>72</v>
+        <v>54</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="E12" s="1">
         <v>654</v>
@@ -1907,42 +1740,28 @@
         <v>2</v>
       </c>
       <c r="M12" s="1">
+        <f t="shared" si="2"/>
         <v>2</v>
       </c>
       <c r="N12" s="1" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="O12" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="P12" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="Q12" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="R12" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="S12" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="T12" s="1" t="s">
-        <v>26</v>
+        <v>55</v>
       </c>
     </row>
-    <row r="13" spans="1:20" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
-        <v>74</v>
+        <v>56</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>75</v>
+        <v>57</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>76</v>
+        <v>58</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="E13" s="1">
         <v>456</v>
@@ -1968,43 +1787,29 @@
         <v>2</v>
       </c>
       <c r="M13" s="1">
+        <f t="shared" si="2"/>
         <v>2</v>
       </c>
       <c r="N13" s="1" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="O13" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="P13" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="Q13" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="R13" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="S13" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="T13" s="1" t="s">
-        <v>26</v>
+        <v>64</v>
       </c>
     </row>
-    <row r="14" spans="1:20" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="str">
         <f>LEFT(A13,4)&amp;TEXT(RIGHT(A13,3)+1,"000")</f>
         <v>JBG-013</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>77</v>
+        <v>59</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>76</v>
+        <v>58</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="E14" s="1">
         <v>145</v>
@@ -2030,43 +1835,29 @@
         <v>2</v>
       </c>
       <c r="M14" s="1">
+        <f t="shared" si="2"/>
         <v>2</v>
       </c>
       <c r="N14" s="1" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="O14" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="P14" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="Q14" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="R14" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="S14" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="T14" s="1" t="s">
-        <v>26</v>
+        <v>66</v>
       </c>
     </row>
-    <row r="15" spans="1:20" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="str">
         <f>LEFT(A14,4)&amp;TEXT(RIGHT(A14,3)+1,"000")</f>
         <v>JBG-014</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>78</v>
+        <v>60</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>81</v>
+        <v>63</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="E15" s="1">
         <v>380</v>
@@ -2092,105 +1883,80 @@
         <v>2</v>
       </c>
       <c r="M15" s="1">
+        <f t="shared" si="2"/>
         <v>2</v>
       </c>
       <c r="N15" s="1" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="O15" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="P15" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="Q15" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="R15" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="S15" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="T15" s="1" t="s">
-        <v>26</v>
+        <v>65</v>
       </c>
     </row>
-    <row r="16" spans="1:20" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="1" t="str">
+    <row r="16" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="5" t="str">
         <f>LEFT(A15,4)&amp;TEXT(RIGHT(A15,3)+1,"000")</f>
         <v>JBG-015</v>
       </c>
-      <c r="B16" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="D16" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="E16" s="1">
+      <c r="B16" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E16" s="5">
         <v>480</v>
       </c>
-      <c r="F16" s="1">
+      <c r="F16" s="5">
         <v>50</v>
       </c>
-      <c r="G16" s="1">
+      <c r="G16" s="5">
         <v>150</v>
       </c>
-      <c r="H16" s="1">
+      <c r="H16" s="5">
         <f t="shared" si="5"/>
         <v>680</v>
       </c>
-      <c r="I16" s="1">
+      <c r="I16" s="5">
         <v>2.5</v>
       </c>
-      <c r="J16" s="1">
+      <c r="J16" s="5">
         <f t="shared" si="6"/>
         <v>1999</v>
       </c>
-      <c r="K16" s="1">
-        <v>2</v>
-      </c>
-      <c r="M16" s="1">
-        <v>2</v>
-      </c>
-      <c r="N16" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="O16" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="P16" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="Q16" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="R16" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="S16" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="T16" s="1" t="s">
-        <v>26</v>
+      <c r="K16" s="5">
+        <v>2</v>
+      </c>
+      <c r="L16" s="5">
+        <v>1</v>
+      </c>
+      <c r="M16" s="5">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="N16" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="O16" s="5" t="s">
+        <v>67</v>
       </c>
     </row>
-    <row r="17" spans="1:20" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="str">
         <f>LEFT(A16,4)&amp;TEXT(RIGHT(A16,3)+1,"000")</f>
         <v>JBG-016</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>80</v>
+        <v>62</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>81</v>
+        <v>63</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="E17" s="1">
         <v>425</v>
@@ -2216,45 +1982,313 @@
         <v>1</v>
       </c>
       <c r="M17" s="1">
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="N17" s="1" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="O17" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="P17" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="Q17" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="R17" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="S17" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="T17" s="1" t="s">
-        <v>26</v>
+        <v>68</v>
       </c>
     </row>
-    <row r="18" spans="1:20" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="19" spans="1:20" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="20" spans="1:20" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="21" spans="1:20" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="22" spans="1:20" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="23" spans="1:20" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="24" spans="1:20" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="25" spans="1:20" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="26" spans="1:20" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="27" spans="1:20" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="28" spans="1:20" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="29" spans="1:20" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="30" spans="1:20" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="31" spans="1:20" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="32" spans="1:20" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="18" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="1" t="str">
+        <f>LEFT(A17,4)&amp;TEXT(RIGHT(A17,3)+1,"000")</f>
+        <v>JBG-017</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E18" s="1">
+        <v>768</v>
+      </c>
+      <c r="F18" s="1">
+        <v>50</v>
+      </c>
+      <c r="G18" s="1">
+        <v>150</v>
+      </c>
+      <c r="H18" s="1">
+        <f t="shared" ref="H18" si="7">SUM(E18:G18)</f>
+        <v>968</v>
+      </c>
+      <c r="I18" s="1">
+        <v>3</v>
+      </c>
+      <c r="J18" s="1">
+        <f t="shared" ref="J18" si="8">ROUNDUP((H18*I18)/500,0)*500-1</f>
+        <v>2999</v>
+      </c>
+      <c r="K18" s="1">
+        <v>2</v>
+      </c>
+      <c r="M18" s="1">
+        <f t="shared" ref="M18" si="9">K18-L18</f>
+        <v>2</v>
+      </c>
+      <c r="N18" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="O18" s="1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="19" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="1" t="str">
+        <f>LEFT(A18,4)&amp;TEXT(RIGHT(A18,3)+1,"000")</f>
+        <v>JBG-018</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E19" s="1">
+        <v>516</v>
+      </c>
+      <c r="F19" s="1">
+        <v>50</v>
+      </c>
+      <c r="G19" s="1">
+        <v>150</v>
+      </c>
+      <c r="H19" s="1">
+        <f t="shared" ref="H19" si="10">SUM(E19:G19)</f>
+        <v>716</v>
+      </c>
+      <c r="I19" s="1">
+        <v>3</v>
+      </c>
+      <c r="J19" s="1">
+        <f t="shared" ref="J19" si="11">ROUNDUP((H19*I19)/500,0)*500-1</f>
+        <v>2499</v>
+      </c>
+      <c r="K19" s="1">
+        <v>2</v>
+      </c>
+      <c r="M19" s="1">
+        <f t="shared" ref="M19" si="12">K19-L19</f>
+        <v>2</v>
+      </c>
+      <c r="N19" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="O19" s="1" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="20" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="1" t="str">
+        <f>LEFT(A19,4)&amp;TEXT(RIGHT(A19,3)+1,"000")</f>
+        <v>JBG-019</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E20" s="1">
+        <v>135</v>
+      </c>
+      <c r="F20" s="1">
+        <v>50</v>
+      </c>
+      <c r="G20" s="1">
+        <v>150</v>
+      </c>
+      <c r="H20" s="1">
+        <f t="shared" ref="H20" si="13">SUM(E20:G20)</f>
+        <v>335</v>
+      </c>
+      <c r="I20" s="1">
+        <v>3</v>
+      </c>
+      <c r="J20" s="1">
+        <f t="shared" ref="J20" si="14">ROUNDUP((H20*I20)/500,0)*500-1</f>
+        <v>1499</v>
+      </c>
+      <c r="K20" s="1">
+        <v>2</v>
+      </c>
+      <c r="M20" s="1">
+        <f t="shared" ref="M20" si="15">K20-L20</f>
+        <v>2</v>
+      </c>
+      <c r="N20" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="O20" s="1" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="21" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="1" t="str">
+        <f>LEFT(A20,4)&amp;TEXT(RIGHT(A20,3)+1,"000")</f>
+        <v>JBG-020</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E21" s="1">
+        <v>135</v>
+      </c>
+      <c r="F21" s="1">
+        <v>50</v>
+      </c>
+      <c r="G21" s="1">
+        <v>150</v>
+      </c>
+      <c r="H21" s="1">
+        <f t="shared" ref="H21" si="16">SUM(E21:G21)</f>
+        <v>335</v>
+      </c>
+      <c r="I21" s="1">
+        <v>3</v>
+      </c>
+      <c r="J21" s="1">
+        <f t="shared" ref="J21" si="17">ROUNDUP((H21*I21)/500,0)*500-1</f>
+        <v>1499</v>
+      </c>
+      <c r="K21" s="1">
+        <v>2</v>
+      </c>
+      <c r="M21" s="1">
+        <f t="shared" ref="M21" si="18">K21-L21</f>
+        <v>2</v>
+      </c>
+      <c r="N21" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="O21" s="1" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="22" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="1" t="str">
+        <f>LEFT(A21,4)&amp;TEXT(RIGHT(A21,3)+1,"000")</f>
+        <v>JBG-021</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E22" s="1">
+        <v>160</v>
+      </c>
+      <c r="F22" s="1">
+        <v>50</v>
+      </c>
+      <c r="G22" s="1">
+        <v>150</v>
+      </c>
+      <c r="H22" s="1">
+        <f t="shared" ref="H22:H23" si="19">SUM(E22:G22)</f>
+        <v>360</v>
+      </c>
+      <c r="I22" s="1">
+        <v>3</v>
+      </c>
+      <c r="J22" s="1">
+        <f t="shared" ref="J22:J23" si="20">ROUNDUP((H22*I22)/500,0)*500-1</f>
+        <v>1499</v>
+      </c>
+      <c r="K22" s="1">
+        <v>2</v>
+      </c>
+      <c r="M22" s="1">
+        <f t="shared" ref="M22:M23" si="21">K22-L22</f>
+        <v>2</v>
+      </c>
+      <c r="N22" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="O22" s="1" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="23" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="1" t="str">
+        <f>LEFT(A22,4)&amp;TEXT(RIGHT(A22,3)+1,"000")</f>
+        <v>JBG-022</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E23" s="1">
+        <v>115</v>
+      </c>
+      <c r="F23" s="1">
+        <v>50</v>
+      </c>
+      <c r="G23" s="1">
+        <v>150</v>
+      </c>
+      <c r="H23" s="1">
+        <f t="shared" si="19"/>
+        <v>315</v>
+      </c>
+      <c r="I23" s="1">
+        <v>3</v>
+      </c>
+      <c r="J23" s="1">
+        <f t="shared" si="20"/>
+        <v>999</v>
+      </c>
+      <c r="K23" s="1">
+        <v>2</v>
+      </c>
+      <c r="M23" s="1">
+        <f t="shared" si="21"/>
+        <v>2</v>
+      </c>
+      <c r="N23" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="O23" s="1" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="24" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="25" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="26" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="27" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="28" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="29" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="30" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="31" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="32" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="33" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="34" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="35" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
@@ -2280,6 +2314,9 @@
     <row r="55" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="56" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
+  <conditionalFormatting sqref="O1:O1048576">
+    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <ignoredErrors>

</xml_diff>

<commit_message>
Add shuffle to featured, add American Diamond category with Adaa/Ruhani/Chandni/Rajsi
</commit_message>
<xml_diff>
--- a/business/inventory-ledger.xlsx
+++ b/business/inventory-ledger.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ahujadiv\Desktop\Team\Automations\JBG\jewels-by-geetika\business\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A717F24C-CD11-42E0-858F-2747C58DCD80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A2AB4CB-51E2-4FB5-8E49-ADB13FC5C6B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{68BF2D20-07EA-4E2C-B5AF-3720521CC247}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{68BF2D20-07EA-4E2C-B5AF-3720521CC247}"/>
   </bookViews>
   <sheets>
     <sheet name="inventory-ledger" sheetId="1" r:id="rId1"/>
+    <sheet name="Box Size" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -33,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="94">
   <si>
     <t>Product ID</t>
   </si>
@@ -279,6 +280,42 @@
   </si>
   <si>
     <t>JBG-ATB-002</t>
+  </si>
+  <si>
+    <t>Box</t>
+  </si>
+  <si>
+    <t>Inches</t>
+  </si>
+  <si>
+    <t>Centimeters</t>
+  </si>
+  <si>
+    <t>Large</t>
+  </si>
+  <si>
+    <t>10 × 7 × 3</t>
+  </si>
+  <si>
+    <t>25 × 18 × 8</t>
+  </si>
+  <si>
+    <t>Medium</t>
+  </si>
+  <si>
+    <t>6 × 4 × 3</t>
+  </si>
+  <si>
+    <t>15 × 10 × 8</t>
+  </si>
+  <si>
+    <t>Small</t>
+  </si>
+  <si>
+    <t>4 × 3 × 2</t>
+  </si>
+  <si>
+    <t>10 × 8 × 5</t>
   </si>
 </sst>
 </file>
@@ -1799,7 +1836,7 @@
     </row>
     <row r="14" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="str">
-        <f>LEFT(A13,4)&amp;TEXT(RIGHT(A13,3)+1,"000")</f>
+        <f t="shared" ref="A14:A23" si="5">LEFT(A13,4)&amp;TEXT(RIGHT(A13,3)+1,"000")</f>
         <v>JBG-013</v>
       </c>
       <c r="B14" s="1" t="s">
@@ -1821,14 +1858,14 @@
         <v>150</v>
       </c>
       <c r="H14" s="1">
-        <f t="shared" ref="H14:H17" si="5">SUM(E14:G14)</f>
+        <f t="shared" ref="H14:H17" si="6">SUM(E14:G14)</f>
         <v>345</v>
       </c>
       <c r="I14" s="1">
         <v>3</v>
       </c>
       <c r="J14" s="1">
-        <f t="shared" ref="J14:J17" si="6">ROUNDUP((H14*I14)/500,0)*500-1</f>
+        <f t="shared" ref="J14:J17" si="7">ROUNDUP((H14*I14)/500,0)*500-1</f>
         <v>1499</v>
       </c>
       <c r="K14" s="1">
@@ -1847,7 +1884,7 @@
     </row>
     <row r="15" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="str">
-        <f>LEFT(A14,4)&amp;TEXT(RIGHT(A14,3)+1,"000")</f>
+        <f t="shared" si="5"/>
         <v>JBG-014</v>
       </c>
       <c r="B15" s="1" t="s">
@@ -1869,14 +1906,14 @@
         <v>150</v>
       </c>
       <c r="H15" s="1">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>580</v>
       </c>
       <c r="I15" s="1">
         <v>2.5</v>
       </c>
       <c r="J15" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>1499</v>
       </c>
       <c r="K15" s="1">
@@ -1895,7 +1932,7 @@
     </row>
     <row r="16" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="5" t="str">
-        <f>LEFT(A15,4)&amp;TEXT(RIGHT(A15,3)+1,"000")</f>
+        <f t="shared" si="5"/>
         <v>JBG-015</v>
       </c>
       <c r="B16" s="5" t="s">
@@ -1917,14 +1954,14 @@
         <v>150</v>
       </c>
       <c r="H16" s="5">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>680</v>
       </c>
       <c r="I16" s="5">
         <v>2.5</v>
       </c>
       <c r="J16" s="5">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>1999</v>
       </c>
       <c r="K16" s="5">
@@ -1946,7 +1983,7 @@
     </row>
     <row r="17" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="str">
-        <f>LEFT(A16,4)&amp;TEXT(RIGHT(A16,3)+1,"000")</f>
+        <f t="shared" si="5"/>
         <v>JBG-016</v>
       </c>
       <c r="B17" s="1" t="s">
@@ -1968,14 +2005,14 @@
         <v>150</v>
       </c>
       <c r="H17" s="1">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>625</v>
       </c>
       <c r="I17" s="1">
         <v>2</v>
       </c>
       <c r="J17" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>1499</v>
       </c>
       <c r="K17" s="1">
@@ -1994,7 +2031,7 @@
     </row>
     <row r="18" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="str">
-        <f>LEFT(A17,4)&amp;TEXT(RIGHT(A17,3)+1,"000")</f>
+        <f t="shared" si="5"/>
         <v>JBG-017</v>
       </c>
       <c r="B18" s="1" t="s">
@@ -2016,21 +2053,21 @@
         <v>150</v>
       </c>
       <c r="H18" s="1">
-        <f t="shared" ref="H18" si="7">SUM(E18:G18)</f>
+        <f t="shared" ref="H18" si="8">SUM(E18:G18)</f>
         <v>968</v>
       </c>
       <c r="I18" s="1">
         <v>3</v>
       </c>
       <c r="J18" s="1">
-        <f t="shared" ref="J18" si="8">ROUNDUP((H18*I18)/500,0)*500-1</f>
+        <f t="shared" ref="J18" si="9">ROUNDUP((H18*I18)/500,0)*500-1</f>
         <v>2999</v>
       </c>
       <c r="K18" s="1">
         <v>2</v>
       </c>
       <c r="M18" s="1">
-        <f t="shared" ref="M18" si="9">K18-L18</f>
+        <f t="shared" ref="M18" si="10">K18-L18</f>
         <v>2</v>
       </c>
       <c r="N18" s="1" t="s">
@@ -2042,7 +2079,7 @@
     </row>
     <row r="19" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="str">
-        <f>LEFT(A18,4)&amp;TEXT(RIGHT(A18,3)+1,"000")</f>
+        <f t="shared" si="5"/>
         <v>JBG-018</v>
       </c>
       <c r="B19" s="1" t="s">
@@ -2064,21 +2101,21 @@
         <v>150</v>
       </c>
       <c r="H19" s="1">
-        <f t="shared" ref="H19" si="10">SUM(E19:G19)</f>
+        <f t="shared" ref="H19" si="11">SUM(E19:G19)</f>
         <v>716</v>
       </c>
       <c r="I19" s="1">
         <v>3</v>
       </c>
       <c r="J19" s="1">
-        <f t="shared" ref="J19" si="11">ROUNDUP((H19*I19)/500,0)*500-1</f>
+        <f t="shared" ref="J19" si="12">ROUNDUP((H19*I19)/500,0)*500-1</f>
         <v>2499</v>
       </c>
       <c r="K19" s="1">
         <v>2</v>
       </c>
       <c r="M19" s="1">
-        <f t="shared" ref="M19" si="12">K19-L19</f>
+        <f t="shared" ref="M19" si="13">K19-L19</f>
         <v>2</v>
       </c>
       <c r="N19" s="1" t="s">
@@ -2090,7 +2127,7 @@
     </row>
     <row r="20" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="str">
-        <f>LEFT(A19,4)&amp;TEXT(RIGHT(A19,3)+1,"000")</f>
+        <f t="shared" si="5"/>
         <v>JBG-019</v>
       </c>
       <c r="B20" s="1" t="s">
@@ -2112,21 +2149,21 @@
         <v>150</v>
       </c>
       <c r="H20" s="1">
-        <f t="shared" ref="H20" si="13">SUM(E20:G20)</f>
+        <f t="shared" ref="H20" si="14">SUM(E20:G20)</f>
         <v>335</v>
       </c>
       <c r="I20" s="1">
         <v>3</v>
       </c>
       <c r="J20" s="1">
-        <f t="shared" ref="J20" si="14">ROUNDUP((H20*I20)/500,0)*500-1</f>
+        <f t="shared" ref="J20" si="15">ROUNDUP((H20*I20)/500,0)*500-1</f>
         <v>1499</v>
       </c>
       <c r="K20" s="1">
         <v>2</v>
       </c>
       <c r="M20" s="1">
-        <f t="shared" ref="M20" si="15">K20-L20</f>
+        <f t="shared" ref="M20" si="16">K20-L20</f>
         <v>2</v>
       </c>
       <c r="N20" s="1" t="s">
@@ -2138,7 +2175,7 @@
     </row>
     <row r="21" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="str">
-        <f>LEFT(A20,4)&amp;TEXT(RIGHT(A20,3)+1,"000")</f>
+        <f t="shared" si="5"/>
         <v>JBG-020</v>
       </c>
       <c r="B21" s="1" t="s">
@@ -2160,21 +2197,21 @@
         <v>150</v>
       </c>
       <c r="H21" s="1">
-        <f t="shared" ref="H21" si="16">SUM(E21:G21)</f>
+        <f t="shared" ref="H21" si="17">SUM(E21:G21)</f>
         <v>335</v>
       </c>
       <c r="I21" s="1">
         <v>3</v>
       </c>
       <c r="J21" s="1">
-        <f t="shared" ref="J21" si="17">ROUNDUP((H21*I21)/500,0)*500-1</f>
+        <f t="shared" ref="J21" si="18">ROUNDUP((H21*I21)/500,0)*500-1</f>
         <v>1499</v>
       </c>
       <c r="K21" s="1">
         <v>2</v>
       </c>
       <c r="M21" s="1">
-        <f t="shared" ref="M21" si="18">K21-L21</f>
+        <f t="shared" ref="M21" si="19">K21-L21</f>
         <v>2</v>
       </c>
       <c r="N21" s="1" t="s">
@@ -2186,7 +2223,7 @@
     </row>
     <row r="22" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="str">
-        <f>LEFT(A21,4)&amp;TEXT(RIGHT(A21,3)+1,"000")</f>
+        <f t="shared" si="5"/>
         <v>JBG-021</v>
       </c>
       <c r="B22" s="1" t="s">
@@ -2208,21 +2245,21 @@
         <v>150</v>
       </c>
       <c r="H22" s="1">
-        <f t="shared" ref="H22:H23" si="19">SUM(E22:G22)</f>
+        <f t="shared" ref="H22:H23" si="20">SUM(E22:G22)</f>
         <v>360</v>
       </c>
       <c r="I22" s="1">
         <v>3</v>
       </c>
       <c r="J22" s="1">
-        <f t="shared" ref="J22:J23" si="20">ROUNDUP((H22*I22)/500,0)*500-1</f>
+        <f t="shared" ref="J22:J23" si="21">ROUNDUP((H22*I22)/500,0)*500-1</f>
         <v>1499</v>
       </c>
       <c r="K22" s="1">
         <v>2</v>
       </c>
       <c r="M22" s="1">
-        <f t="shared" ref="M22:M23" si="21">K22-L22</f>
+        <f t="shared" ref="M22:M23" si="22">K22-L22</f>
         <v>2</v>
       </c>
       <c r="N22" s="1" t="s">
@@ -2234,7 +2271,7 @@
     </row>
     <row r="23" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="str">
-        <f>LEFT(A22,4)&amp;TEXT(RIGHT(A22,3)+1,"000")</f>
+        <f t="shared" si="5"/>
         <v>JBG-022</v>
       </c>
       <c r="B23" s="1" t="s">
@@ -2256,21 +2293,21 @@
         <v>150</v>
       </c>
       <c r="H23" s="1">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>315</v>
       </c>
       <c r="I23" s="1">
         <v>3</v>
       </c>
       <c r="J23" s="1">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>999</v>
       </c>
       <c r="K23" s="1">
         <v>2</v>
       </c>
       <c r="M23" s="1">
-        <f t="shared" si="21"/>
+        <f t="shared" si="22"/>
         <v>2</v>
       </c>
       <c r="N23" s="1" t="s">
@@ -2323,4 +2360,62 @@
     <ignoredError sqref="H13" formula="1"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5F3BB488-5BAD-4C68-B909-33D2B8028147}">
+  <dimension ref="K7:M10"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="12" max="12" width="8.44140625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="7" spans="11:13" x14ac:dyDescent="0.3">
+      <c r="K7" t="s">
+        <v>82</v>
+      </c>
+      <c r="L7" t="s">
+        <v>83</v>
+      </c>
+      <c r="M7" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="8" spans="11:13" x14ac:dyDescent="0.3">
+      <c r="K8" t="s">
+        <v>85</v>
+      </c>
+      <c r="L8" t="s">
+        <v>86</v>
+      </c>
+      <c r="M8" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="9" spans="11:13" x14ac:dyDescent="0.3">
+      <c r="K9" t="s">
+        <v>88</v>
+      </c>
+      <c r="L9" t="s">
+        <v>89</v>
+      </c>
+      <c r="M9" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="10" spans="11:13" x14ac:dyDescent="0.3">
+      <c r="K10" t="s">
+        <v>91</v>
+      </c>
+      <c r="L10" t="s">
+        <v>92</v>
+      </c>
+      <c r="M10" t="s">
+        <v>93</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>